<commit_message>
bug/ Correção na implementação dos obstaculos, e criação de logs
</commit_message>
<xml_diff>
--- a/src/data/resultados.xlsx
+++ b/src/data/resultados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,19 +453,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>98.40000000000001</v>
+        <v>100.7</v>
       </c>
       <c r="C2" t="n">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>348</v>
+        <v>276</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -473,19 +473,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>125.65</v>
+        <v>129.4</v>
       </c>
       <c r="C3" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D3" t="n">
         <v>10</v>
       </c>
       <c r="E3" t="n">
-        <v>348</v>
+        <v>276</v>
       </c>
       <c r="F3" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -493,19 +493,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>142.35</v>
+        <v>146.3</v>
       </c>
       <c r="C4" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D4" t="n">
         <v>10</v>
       </c>
       <c r="E4" t="n">
-        <v>348</v>
+        <v>276</v>
       </c>
       <c r="F4" t="n">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -513,19 +513,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>156.1</v>
+        <v>158.6</v>
       </c>
       <c r="C5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D5" t="n">
         <v>10</v>
       </c>
       <c r="E5" t="n">
-        <v>348</v>
+        <v>276</v>
       </c>
       <c r="F5" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
@@ -533,118 +533,18 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>167.75</v>
+        <v>169.35</v>
       </c>
       <c r="C6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
         <v>10</v>
       </c>
       <c r="E6" t="n">
-        <v>348</v>
+        <v>276</v>
       </c>
       <c r="F6" t="n">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>80.45</v>
-      </c>
-      <c r="C7" t="n">
-        <v>12</v>
-      </c>
-      <c r="D7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E7" t="n">
-        <v>56</v>
-      </c>
-      <c r="F7" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="n">
-        <v>64.09999999999999</v>
-      </c>
-      <c r="C8" t="n">
-        <v>10</v>
-      </c>
-      <c r="D8" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" t="n">
-        <v>52</v>
-      </c>
-      <c r="F8" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="n">
-        <v>58.25</v>
-      </c>
-      <c r="C9" t="n">
-        <v>12</v>
-      </c>
-      <c r="D9" t="n">
-        <v>10</v>
-      </c>
-      <c r="E9" t="n">
-        <v>36</v>
-      </c>
-      <c r="F9" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="n">
-        <v>55.75</v>
-      </c>
-      <c r="C10" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" t="n">
-        <v>10</v>
-      </c>
-      <c r="E10" t="n">
-        <v>16</v>
-      </c>
-      <c r="F10" t="n">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="n">
-        <v>55.3</v>
-      </c>
-      <c r="C11" t="n">
-        <v>10</v>
-      </c>
-      <c r="D11" t="n">
-        <v>10</v>
-      </c>
-      <c r="E11" t="n">
-        <v>16</v>
-      </c>
-      <c r="F11" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>